<commit_message>
29/08/2026 & 30/08/2026 Activity update
</commit_message>
<xml_diff>
--- a/12612645.xlsx
+++ b/12612645.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shash\Desktop\Activities\12612645\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BE94736-FA45-4150-93D4-29E4EE948DD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D56AF0-3EE2-4180-851D-F8B1CE1C3EBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="72">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1579,69 +1579,135 @@
       <c r="N17" s="17"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="8">
+        <v>46263</v>
+      </c>
+      <c r="B18" s="14">
+        <v>240</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D18" s="14">
+        <v>360</v>
+      </c>
+      <c r="E18" s="14">
+        <v>210</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0</v>
+      </c>
+      <c r="H18" s="14">
+        <v>240</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
+        <v>390</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N18" s="17"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="8">
+        <v>46264</v>
+      </c>
+      <c r="B19" s="14">
+        <v>360</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="14">
+        <v>300</v>
+      </c>
+      <c r="E19" s="14">
+        <v>180</v>
+      </c>
+      <c r="F19" s="14">
+        <v>0</v>
+      </c>
+      <c r="G19" s="14">
+        <v>0</v>
+      </c>
+      <c r="H19" s="14">
+        <v>180</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>1020</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
+        <v>420</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N19" s="17"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="A20" s="8">
+        <v>46265</v>
+      </c>
+      <c r="B20" s="14">
+        <v>300</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="14">
+        <v>300</v>
+      </c>
+      <c r="E20" s="14">
+        <v>120</v>
+      </c>
+      <c r="F20" s="14">
+        <v>3</v>
+      </c>
+      <c r="G20" s="14">
+        <v>150</v>
+      </c>
+      <c r="H20" s="14">
+        <v>120</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>843</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
+        <v>597</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>50</v>
+      </c>
       <c r="N20" s="17"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
02/09/2026 and 03/09/2026 Activity update
</commit_message>
<xml_diff>
--- a/12612645.xlsx
+++ b/12612645.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shash\Desktop\Activities\12612645\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA26450-DC32-4027-BB05-5BA04C36F89B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D700208-94CA-4533-AD31-05F754F95892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="72">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1551,21 +1551,21 @@
         <v>180</v>
       </c>
       <c r="F17" s="14">
+        <v>150</v>
+      </c>
+      <c r="G17" s="14">
         <v>3</v>
-      </c>
-      <c r="G17" s="14">
-        <v>150</v>
       </c>
       <c r="H17" s="14">
         <v>150</v>
       </c>
       <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v>1023</v>
+        <v>1170</v>
       </c>
       <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v>417</v>
+        <v>270</v>
       </c>
       <c r="K17" s="16" t="s">
         <v>62</v>
@@ -1683,21 +1683,21 @@
         <v>150</v>
       </c>
       <c r="F20" s="14">
+        <v>150</v>
+      </c>
+      <c r="G20" s="14">
         <v>3</v>
-      </c>
-      <c r="G20" s="14">
-        <v>150</v>
       </c>
       <c r="H20" s="14">
         <v>120</v>
       </c>
       <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v>873</v>
+        <v>1020</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v>567</v>
+        <v>420</v>
       </c>
       <c r="K20" s="16" t="s">
         <v>62</v>
@@ -1727,21 +1727,21 @@
         <v>210</v>
       </c>
       <c r="F21" s="14">
+        <v>200</v>
+      </c>
+      <c r="G21" s="14">
         <v>4</v>
-      </c>
-      <c r="G21" s="14">
-        <v>200</v>
       </c>
       <c r="H21" s="14">
         <v>180</v>
       </c>
       <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v>994</v>
+        <v>1190</v>
       </c>
       <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v>446</v>
+        <v>250</v>
       </c>
       <c r="K21" s="16" t="s">
         <v>62</v>
@@ -1755,47 +1755,91 @@
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="8">
+        <v>46267</v>
+      </c>
+      <c r="B22" s="14">
+        <v>240</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" s="14">
+        <v>360</v>
+      </c>
+      <c r="E22" s="14">
+        <v>180</v>
+      </c>
+      <c r="F22" s="14">
+        <v>150</v>
+      </c>
+      <c r="G22" s="14">
+        <v>3</v>
+      </c>
+      <c r="H22" s="14">
+        <v>150</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
+        <v>360</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N22" s="17"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+    <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="8">
+        <v>46268</v>
+      </c>
+      <c r="B23" s="14">
+        <v>240</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="D23" s="14">
+        <v>300</v>
+      </c>
+      <c r="E23" s="14">
+        <v>240</v>
+      </c>
+      <c r="F23" s="14">
+        <v>200</v>
+      </c>
+      <c r="G23" s="14">
+        <v>4</v>
+      </c>
+      <c r="H23" s="14">
+        <v>240</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>1220</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
+        <v>220</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>60</v>
+      </c>
       <c r="N23" s="17"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>